<commit_message>
GTM: pricing v2 package + Aylık prices confirmed by Atilla (modules still a proposal); ERP tasks and decisions log updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -1916,7 +1916,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Confirm pricing v2 numbers (Başlangıç / Büyüme / Pro / Kurumsal, Aylık, modules)</t>
+          <t>Confirm pricing v2 package prices (Başlangıç / Büyüme / Pro / Kurumsal, Aylık)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1945,7 +1945,7 @@
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Model decided 19 Oct; numbers are a proposal</t>
+          <t>Confirmed 19 Oct 19:48 via command board</t>
         </is>
       </c>
       <c r="J9" s="4">
@@ -1956,12 +1956,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T05b</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Take the 4 accountant questions (seller of record + KDV, partner payout paperwork, deductibility)</t>
+          <t>Confirm pricing v2 module prices (finance, arbitrage, photo studio, extra store/orders)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1990,7 +1990,7 @@
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>pricing-v2 §5. Decides iyzico/PayTR entity</t>
+          <t>Still a proposal</t>
         </is>
       </c>
       <c r="J10" s="4">
@@ -2001,25 +2001,25 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Accountant answers the 4 questions</t>
+          <t>Take the 4 accountant questions (seller of record + KDV, partner payout paperwork, deductibility)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Accountant</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>46333</v>
+        <v>46326</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -2032,12 +2032,12 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>pricing-v2 §5. Decides iyzico/PayTR entity</t>
+        </is>
+      </c>
       <c r="J11" s="4">
         <f>IF(AND(D11&lt;&gt;"",D11&lt;TODAY(),E11&lt;&gt;"Done",E11&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2046,40 +2046,40 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>OK to switch the tutorials Unlisted → Public</t>
+          <t>Accountant answers the 4 questions</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Atilla</t>
+          <t>Accountant</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>46328</v>
+        <v>46333</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com</t>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr"/>
@@ -2091,12 +2091,12 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Create the Stripe partner coupon(s) and set STRIPE_PARTNER_COUPON_ID via stdin</t>
+          <t>OK to switch the tutorials Unlisted → Public</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -2114,20 +2114,20 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://dashboard.stripe.com/coupons</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>20% once on yearly / repeating 3 months on Aylık</t>
-        </is>
-      </c>
+          <t>https://studio.youtube.com</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr"/>
       <c r="J13" s="4">
         <f>IF(AND(D13&lt;&gt;"",D13&lt;TODAY(),E13&lt;&gt;"Done",E13&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2136,12 +2136,12 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Create GTM container + GA4 + Meta pixel IDs and set them in the Hetzner .env</t>
+          <t>Create the Stripe partner coupon(s) and set STRIPE_PARTNER_COUPON_ID via stdin</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>46356</v>
+        <v>46328</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -2164,13 +2164,13 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/tracking/README.md</t>
+          <t>https://dashboard.stripe.com/coupons</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Phase 2 gate</t>
+          <t>20% once on yearly / repeating 3 months on Aylık</t>
         </is>
       </c>
       <c r="J14" s="4">
@@ -2181,12 +2181,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Enable Stripe Global Payouts on the Tamsar, Inc. account</t>
+          <t>Create GTM container + GA4 + Meta pixel IDs and set them in the Hetzner .env</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>46376</v>
+        <v>46356</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
@@ -2204,22 +2204,18 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://dashboard.stripe.com</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/tracking/README.md</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Before the first payout run (5 Jan)</t>
+          <t>Phase 2 gate</t>
         </is>
       </c>
       <c r="J15" s="4">
@@ -2230,12 +2226,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Follow up Hepsiburada integrator ticket 1-404875606841365</t>
+          <t>Enable Stripe Global Payouts on the Tamsar, Inc. account</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -2244,11 +2240,11 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>46316</v>
+        <v>46376</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -2256,11 +2252,19 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://dashboard.stripe.com</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Planned close 21 Oct (Satıcı Paneli › Destek Kayıtlarım)</t>
+          <t>Before the first payout run (5 Jan)</t>
         </is>
       </c>
       <c r="J16" s="4">
@@ -2271,41 +2275,37 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Hire a Bionluk freelancer for list-building (120 groups + 60 X/YouTube)</t>
+          <t>Follow up Hepsiburada integrator ticket 1-404875606841365</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>46322</v>
+        <v>46316</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
-        </is>
-      </c>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Budget ₺4–6k; brief in gameplan §4.4</t>
+          <t>Planned close 21 Oct (Satıcı Paneli › Destek Kayıtlarım)</t>
         </is>
       </c>
       <c r="J17" s="4">
@@ -2316,12 +2316,12 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Shortlist + score 110 FB/Telegram groups and 20 müşavirler in Partner pipeline</t>
+          <t>Hire a Bionluk freelancer for list-building (120 groups + 60 X/YouTube)</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>46325</v>
+        <v>46322</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
@@ -2342,15 +2342,15 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>T13</t>
-        </is>
-      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Scoring rubric: gameplan §4.4</t>
+          <t>Budget ₺4–6k; brief in gameplan §4.4</t>
         </is>
       </c>
       <c r="J18" s="4">
@@ -2361,17 +2361,17 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Shortlist + score 50 X accounts and 20 YouTube channels in Partner pipeline</t>
+          <t>Shortlist + score 110 FB/Telegram groups and 20 müşavirler in Partner pipeline</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Ekin</t>
+          <t>Merisa</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
@@ -2388,8 +2388,16 @@
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="8" t="inlineStr"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Scoring rubric: gameplan §4.4</t>
+        </is>
+      </c>
       <c r="J19" s="4">
         <f>IF(AND(D19&lt;&gt;"",D19&lt;TODAY(),E19&lt;&gt;"Done",E19&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2398,17 +2406,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Week 1: 15 helpful answers in target groups (no links)</t>
+          <t>Shortlist + score 50 X accounts and 20 YouTube channels in Partner pipeline</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
+          <t>Ekin</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
@@ -2421,7 +2429,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
@@ -2435,17 +2443,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Week 1: 15 helpful X replies on e-ihracat threads</t>
+          <t>Week 1: 15 helpful answers in target groups (no links)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Ekin</t>
+          <t>Merisa</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
@@ -2472,21 +2480,21 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>T18</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Manual prod check of referral Stage A: open /?ref=TEST-PARTNER, sign up, see 1 signup in /admin/partners, then delete test data</t>
+          <t>Week 1: 15 helpful X replies on e-ihracat threads</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
+          <t>Ekin</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>46319</v>
+        <v>46325</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
@@ -2495,20 +2503,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>https://kolayxport.com/admin/partners</t>
-        </is>
-      </c>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
       <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>With Claude d7; see Tests Q01</t>
-        </is>
-      </c>
+      <c r="I22" s="8" t="inlineStr"/>
       <c r="J22" s="4">
         <f>IF(AND(D22&lt;&gt;"",D22&lt;TODAY(),E22&lt;&gt;"Done",E22&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2517,12 +2517,12 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Send the first partner messages (Varyant 5 / 6)</t>
+          <t>Manual prod check of referral Stage A: open /?ref=TEST-PARTNER, sign up, see 1 signup in /admin/partners, then delete test data</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>46328</v>
+        <v>46319</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
@@ -2545,17 +2545,13 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>T09, T18</t>
-        </is>
-      </c>
+          <t>https://kolayxport.com/admin/partners</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Only after tracking is confirmed</t>
+          <t>With Claude d7; see Tests Q01</t>
         </is>
       </c>
       <c r="J23" s="4">
@@ -2566,12 +2562,12 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Fact-check the blog posts (2 a week)</t>
+          <t>Send the first partner messages (Varyant 5 / 6)</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2580,7 +2576,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -2589,18 +2585,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>T09, T18</t>
+        </is>
+      </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Recurring every Tue/Thu</t>
+          <t>Only after tracking is confirmed</t>
         </is>
       </c>
       <c r="J24" s="4">
@@ -2611,12 +2611,12 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>First live demo in a partner group (scripted, 30 min)</t>
+          <t>Fact-check the blog posts (2 a week)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>46344</v>
+        <v>46329</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -2637,9 +2637,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Recurring every Tue/Thu</t>
+        </is>
+      </c>
       <c r="J25" s="4">
         <f>IF(AND(D25&lt;&gt;"",D25&lt;TODAY(),E25&lt;&gt;"Done",E25&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2648,12 +2656,12 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Ask the first paying customers for written testimonial consent</t>
+          <t>First live demo in a partner group (scripted, 30 min)</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2662,7 +2670,7 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>46365</v>
+        <v>46344</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
@@ -2671,14 +2679,10 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/legal-notes.md</t>
-        </is>
-      </c>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="8" t="inlineStr"/>
       <c r="J26" s="4">
@@ -2689,21 +2693,21 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Phase 2: start Instagram organic (only if the gate passed)</t>
+          <t>Ask the first paying customers for written testimonial consent</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Ekin</t>
+          <t>Merisa</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>46398</v>
+        <v>46365</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -2717,14 +2721,10 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/calendar-30d.md</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Gate</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/legal-notes.md</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="8" t="inlineStr"/>
       <c r="J27" s="4">
         <f>IF(AND(D27&lt;&gt;"",D27&lt;TODAY(),E27&lt;&gt;"Done",E27&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -2734,43 +2734,43 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T23</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Referral Stage A (capture, claim, admin report)</t>
+          <t>Phase 2: start Instagram organic (only if the gate passed)</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Claude: d7 (dev)</t>
+          <t>Ekin</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>46314</v>
+        <v>46398</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>Deployed b6ee9895</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/calendar-30d.md</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr"/>
       <c r="J28" s="4">
         <f>IF(AND(D28&lt;&gt;"",D28&lt;TODAY(),E28&lt;&gt;"Done",E28&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2779,12 +2779,12 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Referral Stage B (bounty ledger, /app/ortaklik, Stripe Global Payouts)</t>
+          <t>Referral Stage A (capture, claim, admin report)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2793,11 +2793,11 @@
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>46333</v>
+        <v>46314</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2810,14 +2810,10 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>T09</t>
-        </is>
-      </c>
+      <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Spec §3–6</t>
+          <t>Deployed b6ee9895</t>
         </is>
       </c>
       <c r="J29" s="4">
@@ -2828,25 +2824,25 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P1: plan keys, yearly limits, modules</t>
+          <t>Referral Stage B (bounty ledger, /app/ortaklik, Stripe Global Payouts)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Claude: to assign</t>
+          <t>Claude: d7 (dev)</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>46341</v>
+        <v>46333</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -2856,15 +2852,19 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>T05</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="inlineStr"/>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>Spec §3–6</t>
+        </is>
+      </c>
       <c r="J30" s="4">
         <f>IF(AND(D30&lt;&gt;"",D30&lt;TODAY(),E30&lt;&gt;"Done",E30&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2873,12 +2873,12 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P2: iyzico/PayTR yearly checkout with taksit</t>
+          <t>Pricing v2 P1: plan keys, yearly limits, modules</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2887,11 +2887,11 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>46356</v>
+        <v>46341</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2906,10 +2906,14 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>T07</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="inlineStr"/>
+          <t>T05b (modules only)</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>Package prices decided; can start</t>
+        </is>
+      </c>
       <c r="J31" s="4">
         <f>IF(AND(D31&lt;&gt;"",D31&lt;TODAY(),E31&lt;&gt;"Done",E31&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2918,17 +2922,17 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P4: /fiyatlandirma redesign</t>
+          <t>Pricing v2 P2: iyzico/PayTR yearly checkout with taksit</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Claude: gtm-overhaul</t>
+          <t>Claude: to assign</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
@@ -2941,7 +2945,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2951,7 +2955,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>T05, T07</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr"/>
@@ -2963,12 +2967,12 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Upload the remaining 8 tutorials</t>
+          <t>Pricing v2 P4: /fiyatlandirma redesign</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2977,11 +2981,11 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>46315</v>
+        <v>46356</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2991,10 +2995,14 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr"/>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>T05, T07</t>
+        </is>
+      </c>
       <c r="I33" s="8" t="inlineStr"/>
       <c r="J33" s="4">
         <f>IF(AND(D33&lt;&gt;"",D33&lt;TODAY(),E33&lt;&gt;"Done",E33&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -3004,12 +3012,12 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Blog cadence: 2 posts a week from the content calendar</t>
+          <t>Upload the remaining 8 tutorials</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3018,11 +3026,11 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>46329</v>
+        <v>46315</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -3032,14 +3040,10 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>T20</t>
-        </is>
-      </c>
+          <t>https://studio.youtube.com</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="8" t="inlineStr"/>
       <c r="J34" s="4">
         <f>IF(AND(D34&lt;&gt;"",D34&lt;TODAY(),E34&lt;&gt;"Done",E34&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -3049,12 +3053,12 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Draft the /ortaklik partner-terms page (publish after Stage B + accountant)</t>
+          <t>Blog cadence: 2 posts a week from the content calendar</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3063,7 +3067,7 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>46333</v>
+        <v>46329</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
@@ -3077,12 +3081,12 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>T07, T25</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="I35" s="8" t="inlineStr"/>
@@ -3094,12 +3098,12 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Privacy notice: one line on masked referrals shown to partners</t>
+          <t>Draft the /ortaklik partner-terms page (publish after Stage B + accountant)</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3122,30 +3126,60 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="8" t="inlineStr">
-        <is>
-          <t>Lawyer-review flag</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>T07, T25</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr"/>
       <c r="J36" s="4">
         <f>IF(AND(D36&lt;&gt;"",D36&lt;TODAY(),E36&lt;&gt;"Done",E36&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
-      <c r="I37" s="8" t="n"/>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>T32</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Privacy notice: one line on masked referrals shown to partners</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Claude: gtm-overhaul</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>46333</v>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>Lawyer-review flag</t>
+        </is>
+      </c>
       <c r="J37" s="4">
         <f>IF(AND(D37&lt;&gt;"",D37&lt;TODAY(),E37&lt;&gt;"Done",E37&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -30203,7 +30237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30511,7 +30545,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Payments collected by Tamsar, Inc. (US) in TRY under its agreement with Modsons</t>
+          <t>Pricing v2 prices CONFIRMED: Başlangıç ₺29.990, Büyüme ₺54.990, Pro ₺89.990, Kurumsal from ₺149.990 a year; Aylık ₺2.999 a month; all +KDV. Module prices still a proposal; partners quote no prices until checkout exists</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -30521,12 +30555,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>pricing-v2 §1</t>
+          <t>command board 19 Oct 19:48 (via orchestrator)</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Proposal: Modsons sells to Turkish customers; open with the accountant</t>
+          <t>Seller of record / KDV still with the accountant</t>
         </is>
       </c>
     </row>
@@ -30536,27 +30570,45 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
+          <t>Payments collected by Tamsar, Inc. (US) in TRY under its agreement with Modsons</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Atilla</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>pricing-v2 §1</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Proposal: Modsons sells to Turkish customers; open with the accountant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
           <t>Cookie panel is live (since 2026-10-17); only tracking IDs gate Phase 2 measurement</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>gtm-overhaul (verified)</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>turkey-gameplan §4.9</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
+      <c r="E18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -30907,6 +30959,13 @@
       <c r="C68" s="4" t="n"/>
       <c r="D68" s="8" t="n"/>
       <c r="E68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="4" t="n"/>
+      <c r="D69" s="8" t="n"/>
+      <c r="E69" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GTM: pricing v2 P1 done (d44c426e, flag off); P3 Stripe prices on hold for the accountant; ERP updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -2883,15 +2883,15 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Claude: to assign</t>
+          <t>Claude: d7 (dev)</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>46341</v>
+        <v>46314</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2904,14 +2904,10 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>T05b (modules only)</t>
-        </is>
-      </c>
+      <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Package prices decided; can start</t>
+          <t>Deployed d44c426e behind PRICING_V2 (flag off)</t>
         </is>
       </c>
       <c r="J31" s="4">
@@ -2922,35 +2918,35 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T26b</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P2: iyzico/PayTR yearly checkout with taksit</t>
+          <t>Pricing v2 P3: Stripe prices for Aylık + modules</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Claude: to assign</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>46356</v>
+        <v>46340</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
+          <t>https://dashboard.stripe.com/products</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2958,7 +2954,11 @@
           <t>T07</t>
         </is>
       </c>
-      <c r="I32" s="8" t="inlineStr"/>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>On hold until the accountant answers (orchestrator decision)</t>
+        </is>
+      </c>
       <c r="J32" s="4">
         <f>IF(AND(D32&lt;&gt;"",D32&lt;TODAY(),E32&lt;&gt;"Done",E32&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2967,17 +2967,17 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P4: /fiyatlandirma redesign</t>
+          <t>Pricing v2 P2: iyzico/PayTR yearly checkout with taksit</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Claude: gtm-overhaul</t>
+          <t>Claude: to assign</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>T05, T07</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr"/>
@@ -3012,12 +3012,12 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Upload the remaining 8 tutorials</t>
+          <t>Pricing v2 P4: /fiyatlandirma redesign</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3026,11 +3026,11 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>46315</v>
+        <v>46356</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -3040,10 +3040,14 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr"/>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>T05, T07</t>
+        </is>
+      </c>
       <c r="I34" s="8" t="inlineStr"/>
       <c r="J34" s="4">
         <f>IF(AND(D34&lt;&gt;"",D34&lt;TODAY(),E34&lt;&gt;"Done",E34&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -3053,12 +3057,12 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Blog cadence: 2 posts a week from the content calendar</t>
+          <t>Upload the remaining 8 tutorials</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3067,11 +3071,11 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>46329</v>
+        <v>46315</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -3081,14 +3085,10 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>T20</t>
-        </is>
-      </c>
+          <t>https://studio.youtube.com</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="8" t="inlineStr"/>
       <c r="J35" s="4">
         <f>IF(AND(D35&lt;&gt;"",D35&lt;TODAY(),E35&lt;&gt;"Done",E35&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -3098,12 +3098,12 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Draft the /ortaklik partner-terms page (publish after Stage B + accountant)</t>
+          <t>Blog cadence: 2 posts a week from the content calendar</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>46333</v>
+        <v>46329</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
@@ -3126,12 +3126,12 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>T07, T25</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="I36" s="8" t="inlineStr"/>
@@ -3143,12 +3143,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Privacy notice: one line on masked referrals shown to partners</t>
+          <t>Draft the /ortaklik partner-terms page (publish after Stage B + accountant)</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3171,30 +3171,60 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="8" t="inlineStr">
-        <is>
-          <t>Lawyer-review flag</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>T07, T25</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr"/>
       <c r="J37" s="4">
         <f>IF(AND(D37&lt;&gt;"",D37&lt;TODAY(),E37&lt;&gt;"Done",E37&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="8" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="8" t="n"/>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>T32</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Privacy notice: one line on masked referrals shown to partners</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Claude: gtm-overhaul</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>46333</v>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Lawyer-review flag</t>
+        </is>
+      </c>
       <c r="J38" s="4">
         <f>IF(AND(D38&lt;&gt;"",D38&lt;TODAY(),E38&lt;&gt;"Done",E38&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>

</xml_diff>

<commit_message>
GTM: Tamsar, Inc. is seller of record, no KDV added (supersedes +KDV); 14 Stripe prices created; iyzico/PayTR dropped, taksit proposed as yearly paid monthly; ERP updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Confirm pricing v2 module prices (finance, arbitrage, photo studio, extra store/orders)</t>
+          <t>Final OK on module prices (finance ₺990, arbitrage ₺990, photo studio ₺790, extra store ₺490, +500 orders ₺490 a month)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1970,11 +1970,11 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>46326</v>
+        <v>46319</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1990,7 +1990,7 @@
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Still a proposal</t>
+          <t>Already created in Stripe at these amounts by d7; on Atilla's board</t>
         </is>
       </c>
       <c r="J10" s="4">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Take the 4 accountant questions (seller of record + KDV, partner payout paperwork, deductibility)</t>
+          <t>Decide seller of record + KDV</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2015,11 +2015,11 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>46326</v>
+        <v>46314</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -2035,7 +2035,7 @@
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>pricing-v2 §5. Decides iyzico/PayTR entity</t>
+          <t>Resolved by Atilla: Tamsar, Inc. sells, TRY via Stripe, no KDV added; Modsons invoices Tamsar</t>
         </is>
       </c>
       <c r="J11" s="4">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Accountant answers the 4 questions</t>
+          <t>Accountant: confirm partner payout paperwork once (W-8BEN; partners declare income in Turkey)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2060,16 +2060,16 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>46333</v>
+        <v>46376</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -2077,12 +2077,12 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Seller question resolved by Atilla (19 Oct); only this check remains, before the first payout (5 Jan)</t>
+        </is>
+      </c>
       <c r="J12" s="4">
         <f>IF(AND(D12&lt;&gt;"",D12&lt;TODAY(),E12&lt;&gt;"Done",E12&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2257,11 +2257,7 @@
           <t>https://dashboard.stripe.com</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
+      <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>Before the first payout run (5 Jan)</t>
@@ -2923,20 +2919,20 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P3: Stripe prices for Aylık + modules</t>
+          <t>Pricing v2 P3: Stripe prices (all 14: yearly packages, Aylık, modules)</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Atilla</t>
+          <t>Claude: d7 (dev)</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>46340</v>
+        <v>46314</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -2949,14 +2945,10 @@
           <t>https://dashboard.stripe.com/products</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
+      <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>On hold until the accountant answers (orchestrator decision)</t>
+          <t>Created live, inert behind PRICING_V2; code waiting for a deploy slot</t>
         </is>
       </c>
       <c r="J32" s="4">
@@ -2972,20 +2964,20 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P2: iyzico/PayTR yearly checkout with taksit</t>
+          <t>Approve taksit option: 'yearly, paid monthly on a 12-month commitment' via Stripe (iyzico/PayTR dropped: Turkish merchants only)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Claude: to assign</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>46356</v>
+        <v>46321</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2998,12 +2990,12 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
-      <c r="I33" s="8" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>pricing-v2 §5; then 3 more Stripe prices + commitment rule (dev)</t>
+        </is>
+      </c>
       <c r="J33" s="4">
         <f>IF(AND(D33&lt;&gt;"",D33&lt;TODAY(),E33&lt;&gt;"Done",E33&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -3017,7 +3009,7 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P4: /fiyatlandirma redesign</t>
+          <t>Pricing v2 P4: /fiyatlandirma redesign (final amounts, no '+KDV')</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3030,7 +3022,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -3045,7 +3037,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>T05, T07</t>
+          <t>T05b, T27</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr"/>
@@ -30267,7 +30259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30625,41 +30617,91 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
+          <t>Seller of record = Tamsar, Inc. for all customers; charges in TRY via Stripe with NO KDV added; prices are final amounts. Modsons invoices Tamsar for services and runs marketing in Turkey</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Atilla</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>d7 session (via orchestrator)</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Supersedes '+KDV' and the Modsons-sells proposal</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>All 14 Stripe prices created (yearly packages, Aylık, modules), live but inert behind PRICING_V2</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Atilla / d7</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>orchestrator</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>iyzico/PayTR dropped (Turkish merchants only; Tamsar, Inc. sells). Taksit replacement proposed: yearly paid monthly on a 12-month commitment</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Plan (proposal)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>pricing-v2 §5</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Waiting for Atilla (T27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
           <t>Cookie panel is live (since 2026-10-17); only tracking IDs gate Phase 2 measurement</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>gtm-overhaul (verified)</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>turkey-gameplan §4.9</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
+      <c r="E21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -30996,6 +31038,27 @@
       <c r="C69" s="4" t="n"/>
       <c r="D69" s="8" t="n"/>
       <c r="E69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="4" t="n"/>
+      <c r="D70" s="8" t="n"/>
+      <c r="E70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n"/>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="4" t="n"/>
+      <c r="D71" s="8" t="n"/>
+      <c r="E71" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n"/>
+      <c r="B72" s="8" t="n"/>
+      <c r="C72" s="4" t="n"/>
+      <c r="D72" s="8" t="n"/>
+      <c r="E72" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GTM: yearly packages pay-in-full only (no taksit, no yearly-paid-monthly), iyzico/PayTR dropped, real taksit parked; docs + ERP updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -2964,7 +2964,7 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Approve taksit option: 'yearly, paid monthly on a 12-month commitment' via Stripe (iyzico/PayTR dropped: Turkish merchants only)</t>
+          <t>Decide taksit option</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2973,11 +2973,11 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2993,7 +2993,7 @@
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>pricing-v2 §5; then 3 more Stripe prices + commitment rule (dev)</t>
+          <t>Decided: yearly = pay-in-full only (Stripe card); Aylık = no-commitment option; iyzico/PayTR dropped. Parked: real taksit only via a Turkish seller entity later</t>
         </is>
       </c>
       <c r="J33" s="4">
@@ -30259,7 +30259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30688,27 +30688,45 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
+          <t>Yearly packages are PAY-IN-FULL ONLY (Stripe card); no 'yearly, paid monthly'; Aylık ₺2.999 stays the no-commitment option; bounty stays 25% of the first yearly payment (no split); P2 iyzico/PayTR dropped</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Atilla</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>board (via orchestrator)</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Parked idea: real taksit only via a Turkish seller entity later</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
           <t>Cookie panel is live (since 2026-10-17); only tracking IDs gate Phase 2 measurement</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>gtm-overhaul (verified)</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>turkey-gameplan §4.9</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
+      <c r="E22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -31059,6 +31077,13 @@
       <c r="C72" s="4" t="n"/>
       <c r="D72" s="8" t="n"/>
       <c r="E72" s="8" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n"/>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="4" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GTM: module prices confirmed by Atilla (19 Oct 20:23); pricing v2 fully decided; ERP updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -1970,11 +1970,11 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1990,7 +1990,7 @@
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Already created in Stripe at these amounts by d7; on Atilla's board</t>
+          <t>Confirmed 19 Oct 20:23 via board; yearly ×10; no KDV added</t>
         </is>
       </c>
       <c r="J10" s="4">
@@ -30259,7 +30259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30713,27 +30713,41 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
+          <t>Module prices CONFIRMED: Finans ₺990, Arbitraj ₺990, Toplu fotoğraf stüdyosu ₺790, Ek mağaza ₺490, +500 sipariş ₺490 a month; yearly ×10; final amounts, no KDV added</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Atilla</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>board 19 Oct 20:23 (via orchestrator)</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
           <t>Cookie panel is live (since 2026-10-17); only tracking IDs gate Phase 2 measurement</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>gtm-overhaul (verified)</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>turkey-gameplan §4.9</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
+      <c r="E23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -31084,6 +31098,13 @@
       <c r="C73" s="4" t="n"/>
       <c r="D73" s="8" t="n"/>
       <c r="E73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="8" t="n"/>
+      <c r="C74" s="4" t="n"/>
+      <c r="D74" s="8" t="n"/>
+      <c r="E74" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GTM ERP: T09 partner coupon done (KX_PARTNER_20_3M)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -2141,20 +2141,20 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Create the Stripe partner coupon(s) and set STRIPE_PARTNER_COUPON_ID via stdin</t>
+          <t>Partner coupon in Stripe + STRIPE_PARTNER_COUPON_ID</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Atilla</t>
+          <t>Claude: d7 (dev)</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>46328</v>
+        <v>46314</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -2170,7 +2170,7 @@
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>20% once on yearly / repeating 3 months on Aylık</t>
+          <t>KX_PARTNER_20_3M: 20% repeating 3 months = 20% once on yearly, first 3 months on Aylık; in prod .env; never stacks with founding</t>
         </is>
       </c>
       <c r="J14" s="4">

</xml_diff>

<commit_message>
GTM ERP: tracking set up (GTM-N6SW5T7K + GA4 G-V4ZC6HS65N on kolayxport@gmail.com), remaining .env + Meta tasks, links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gtm/KolayXport-ERP.xlsx
+++ b/docs/gtm/KolayXport-ERP.xlsx
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Create GTM container + GA4 + Meta pixel IDs and set them in the Hetzner .env</t>
+          <t>Tracking: GTM + GA4 created and published (GTM-N6SW5T7K, G-V4ZC6HS65N, account kolayxport@gmail.com). Remaining: put both IDs in the Hetzner .env + rebuild; mark sign_up/start_trial/purchase as GA4 key events after first data</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -2215,7 +2215,7 @@
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Phase 2 gate</t>
+          <t>Claude set up GTM/GA4 on 19 Oct; .env write is blocked for Claude by permissions</t>
         </is>
       </c>
       <c r="J15" s="4">
@@ -2226,12 +2226,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T10b</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Enable Stripe Global Payouts on the Tamsar, Inc. account</t>
+          <t>Meta pixel + Conversions API token: log in to Meta Business (kolayxport) so it can be created; add the pixel tag in GTM</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>46376</v>
+        <v>46371</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -2249,18 +2249,18 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>https://dashboard.stripe.com</t>
+          <t>https://business.facebook.com/events_manager2</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Before the first payout run (5 Jan)</t>
+          <t>Phase 2 only (ads); Claude cannot enter the Facebook password</t>
         </is>
       </c>
       <c r="J16" s="4">
@@ -2271,12 +2271,12 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Follow up Hepsiburada integrator ticket 1-404875606841365</t>
+          <t>Enable Stripe Global Payouts on the Tamsar, Inc. account</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2285,11 +2285,11 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>46316</v>
+        <v>46376</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2297,11 +2297,15 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>https://dashboard.stripe.com</t>
+        </is>
+      </c>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Planned close 21 Oct (Satıcı Paneli › Destek Kayıtlarım)</t>
+          <t>Before the first payout run (5 Jan)</t>
         </is>
       </c>
       <c r="J17" s="4">
@@ -2312,41 +2316,37 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Hire a Bionluk freelancer for list-building (120 groups + 60 X/YouTube)</t>
+          <t>Follow up Hepsiburada integrator ticket 1-404875606841365</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>46322</v>
+        <v>46316</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
-        </is>
-      </c>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Budget ₺4–6k; brief in gameplan §4.4</t>
+          <t>Planned close 21 Oct (Satıcı Paneli › Destek Kayıtlarım)</t>
         </is>
       </c>
       <c r="J18" s="4">
@@ -2357,12 +2357,12 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Shortlist + score 110 FB/Telegram groups and 20 müşavirler in Partner pipeline</t>
+          <t>Hire a Bionluk freelancer for list-building (120 groups + 60 X/YouTube)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>46325</v>
+        <v>46322</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -2383,15 +2383,15 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>T13</t>
-        </is>
-      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Scoring rubric: gameplan §4.4</t>
+          <t>Budget ₺4–6k; brief in gameplan §4.4</t>
         </is>
       </c>
       <c r="J19" s="4">
@@ -2402,17 +2402,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Shortlist + score 50 X accounts and 20 YouTube channels in Partner pipeline</t>
+          <t>Shortlist + score 110 FB/Telegram groups and 20 müşavirler in Partner pipeline</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Ekin</t>
+          <t>Merisa</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
@@ -2429,8 +2429,16 @@
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="8" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Scoring rubric: gameplan §4.4</t>
+        </is>
+      </c>
       <c r="J20" s="4">
         <f>IF(AND(D20&lt;&gt;"",D20&lt;TODAY(),E20&lt;&gt;"Done",E20&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2439,17 +2447,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Week 1: 15 helpful answers in target groups (no links)</t>
+          <t>Shortlist + score 50 X accounts and 20 YouTube channels in Partner pipeline</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
+          <t>Ekin</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
@@ -2462,7 +2470,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
@@ -2476,17 +2484,17 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Week 1: 15 helpful X replies on e-ihracat threads</t>
+          <t>Week 1: 15 helpful answers in target groups (no links)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Ekin</t>
+          <t>Merisa</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
@@ -2513,21 +2521,21 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>T18</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Manual prod check of referral Stage A: open /?ref=TEST-PARTNER, sign up, see 1 signup in /admin/partners, then delete test data</t>
+          <t>Week 1: 15 helpful X replies on e-ihracat threads</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
+          <t>Ekin</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>46319</v>
+        <v>46325</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
@@ -2536,20 +2544,12 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>https://kolayxport.com/admin/partners</t>
-        </is>
-      </c>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>With Claude d7; see Tests Q01</t>
-        </is>
-      </c>
+      <c r="I23" s="8" t="inlineStr"/>
       <c r="J23" s="4">
         <f>IF(AND(D23&lt;&gt;"",D23&lt;TODAY(),E23&lt;&gt;"Done",E23&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2558,12 +2558,12 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Send the first partner messages (Varyant 5 / 6)</t>
+          <t>Manual prod check of referral Stage A: open /?ref=TEST-PARTNER, sign up, see 1 signup in /admin/partners, then delete test data</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2572,7 +2572,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>46328</v>
+        <v>46319</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -2586,17 +2586,13 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>T09, T18</t>
-        </is>
-      </c>
+          <t>https://kolayxport.com/admin/partners</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Only after tracking is confirmed</t>
+          <t>With Claude d7; see Tests Q01</t>
         </is>
       </c>
       <c r="J24" s="4">
@@ -2607,12 +2603,12 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Fact-check the blog posts (2 a week)</t>
+          <t>Send the first partner messages (Varyant 5 / 6)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2621,7 +2617,7 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -2630,18 +2626,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>T09, T18</t>
+        </is>
+      </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Recurring every Tue/Thu</t>
+          <t>Only after tracking is confirmed</t>
         </is>
       </c>
       <c r="J25" s="4">
@@ -2652,12 +2652,12 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>First live demo in a partner group (scripted, 30 min)</t>
+          <t>Fact-check the blog posts (2 a week)</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>46344</v>
+        <v>46329</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
@@ -2678,9 +2678,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Recurring every Tue/Thu</t>
+        </is>
+      </c>
       <c r="J26" s="4">
         <f>IF(AND(D26&lt;&gt;"",D26&lt;TODAY(),E26&lt;&gt;"Done",E26&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2689,12 +2697,12 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Ask the first paying customers for written testimonial consent</t>
+          <t>First live demo in a partner group (scripted, 30 min)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2703,7 +2711,7 @@
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>46365</v>
+        <v>46344</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -2712,14 +2720,10 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/legal-notes.md</t>
-        </is>
-      </c>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="8" t="inlineStr"/>
       <c r="J27" s="4">
@@ -2730,21 +2734,21 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Phase 2: start Instagram organic (only if the gate passed)</t>
+          <t>Ask the first paying customers for written testimonial consent</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Ekin</t>
+          <t>Merisa</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>46398</v>
+        <v>46365</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
@@ -2758,14 +2762,10 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/calendar-30d.md</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Gate</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/legal-notes.md</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="8" t="inlineStr"/>
       <c r="J28" s="4">
         <f>IF(AND(D28&lt;&gt;"",D28&lt;TODAY(),E28&lt;&gt;"Done",E28&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -2775,43 +2775,43 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T23</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Referral Stage A (capture, claim, admin report)</t>
+          <t>Phase 2: start Instagram organic (only if the gate passed)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Claude: d7 (dev)</t>
+          <t>Ekin</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>46314</v>
+        <v>46398</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>Deployed b6ee9895</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/social/calendar-30d.md</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr"/>
       <c r="J29" s="4">
         <f>IF(AND(D29&lt;&gt;"",D29&lt;TODAY(),E29&lt;&gt;"Done",E29&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -2820,12 +2820,12 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Referral Stage B (bounty ledger, /app/ortaklik, Stripe Global Payouts)</t>
+          <t>Referral Stage A (capture, claim, admin report)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2834,11 +2834,11 @@
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>46333</v>
+        <v>46314</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -2851,14 +2851,10 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>T09</t>
-        </is>
-      </c>
+      <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>Spec §3–6</t>
+          <t>Deployed b6ee9895</t>
         </is>
       </c>
       <c r="J30" s="4">
@@ -2869,12 +2865,12 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P1: plan keys, yearly limits, modules</t>
+          <t>Referral Stage B (bounty ledger, /app/ortaklik, Stripe Global Payouts)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2883,11 +2879,11 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>46314</v>
+        <v>46333</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2897,13 +2893,17 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr"/>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Deployed d44c426e behind PRICING_V2 (flag off)</t>
+          <t>Spec §3–6</t>
         </is>
       </c>
       <c r="J31" s="4">
@@ -2914,12 +2914,12 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>T26b</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P3: Stripe prices (all 14: yearly packages, Aylık, modules)</t>
+          <t>Pricing v2 P1: plan keys, yearly limits, modules</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2937,18 +2937,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>https://dashboard.stripe.com/products</t>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>Created live, inert behind PRICING_V2; code waiting for a deploy slot</t>
+          <t>Deployed d44c426e behind PRICING_V2 (flag off)</t>
         </is>
       </c>
       <c r="J32" s="4">
@@ -2959,17 +2959,17 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T26b</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Decide taksit option</t>
+          <t>Pricing v2 P3: Stripe prices (all 14: yearly packages, Aylık, modules)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Atilla</t>
+          <t>Claude: d7 (dev)</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
@@ -2982,18 +2982,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
+          <t>https://dashboard.stripe.com/products</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Decided: yearly = pay-in-full only (Stripe card); Aylık = no-commitment option; iyzico/PayTR dropped. Parked: real taksit only via a Turkish seller entity later</t>
+          <t>Created live, inert behind PRICING_V2; code waiting for a deploy slot</t>
         </is>
       </c>
       <c r="J33" s="4">
@@ -3004,30 +3004,30 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Pricing v2 P4: /fiyatlandirma redesign (final amounts, no '+KDV')</t>
+          <t>Decide taksit option</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Claude: gtm-overhaul</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>46356</v>
+        <v>46314</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -3035,12 +3035,12 @@
           <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>T05b, T27</t>
-        </is>
-      </c>
-      <c r="I34" s="8" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr"/>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Decided: yearly = pay-in-full only (Stripe card); Aylık = no-commitment option; iyzico/PayTR dropped. Parked: real taksit only via a Turkish seller entity later</t>
+        </is>
+      </c>
       <c r="J34" s="4">
         <f>IF(AND(D34&lt;&gt;"",D34&lt;TODAY(),E34&lt;&gt;"Done",E34&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -3049,12 +3049,12 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Upload the remaining 8 tutorials</t>
+          <t>Pricing v2 P4: /fiyatlandirma redesign (final amounts, no '+KDV')</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3063,11 +3063,11 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>46315</v>
+        <v>46356</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -3077,10 +3077,14 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr"/>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/pricing-v2.md</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>T05b, T27</t>
+        </is>
+      </c>
       <c r="I35" s="8" t="inlineStr"/>
       <c r="J35" s="4">
         <f>IF(AND(D35&lt;&gt;"",D35&lt;TODAY(),E35&lt;&gt;"Done",E35&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -3090,12 +3094,12 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Blog cadence: 2 posts a week from the content calendar</t>
+          <t>Upload the remaining 8 tutorials</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3104,11 +3108,11 @@
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>46329</v>
+        <v>46315</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -3118,14 +3122,10 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>T20</t>
-        </is>
-      </c>
+          <t>https://studio.youtube.com</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="8" t="inlineStr"/>
       <c r="J36" s="4">
         <f>IF(AND(D36&lt;&gt;"",D36&lt;TODAY(),E36&lt;&gt;"Done",E36&lt;&gt;"Cancelled"),"OVERDUE","")</f>
@@ -3135,12 +3135,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Draft the /ortaklik partner-terms page (publish after Stage B + accountant)</t>
+          <t>Blog cadence: 2 posts a week from the content calendar</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>46333</v>
+        <v>46329</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
@@ -3163,12 +3163,12 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/seo/content-calendar.md</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>T07, T25</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr"/>
@@ -3180,12 +3180,12 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Privacy notice: one line on masked referrals shown to partners</t>
+          <t>Draft the /ortaklik partner-terms page (publish after Stage B + accountant)</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -3208,30 +3208,60 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="8" t="inlineStr">
-        <is>
-          <t>Lawyer-review flag</t>
-        </is>
-      </c>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/turkey-gameplan.md</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>T07, T25</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr"/>
       <c r="J38" s="4">
         <f>IF(AND(D38&lt;&gt;"",D38&lt;TODAY(),E38&lt;&gt;"Done",E38&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="8" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
-      <c r="I39" s="8" t="n"/>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>T32</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Privacy notice: one line on masked referrals shown to partners</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Claude: gtm-overhaul</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>46333</v>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/bloodyteeths/kolayxport_supa/blob/main/docs/gtm/referral-spec.md</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>Lawyer-review flag</t>
+        </is>
+      </c>
       <c r="J39" s="4">
         <f>IF(AND(D39&lt;&gt;"",D39&lt;TODAY(),E39&lt;&gt;"Done",E39&lt;&gt;"Cancelled"),"OVERDUE","")</f>
         <v/>
@@ -29314,7 +29344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -29888,20 +29918,24 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>YouTube Studio</t>
+          <t>Google Tag Manager (GTM-N6SW5T7K)</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com</t>
+          <t>https://tagmanager.google.com/?authuser=kolayxport@gmail.com#/container/accounts/6383523253/containers/267664935/workspaces/2</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Atilla</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr"/>
+          <t>Atilla, Merisa</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Account KolayXport (Tamsar, Inc.) on kolayxport@gmail.com; v2 published 19 Oct</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -29911,22 +29945,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Stripe dashboard (Tamsar, Inc.)</t>
+          <t>Google Analytics 4 (G-V4ZC6HS65N)</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>https://dashboard.stripe.com</t>
+          <t>https://analytics.google.com/analytics/web/?authuser=kolayxport@gmail.com#/a412601386p559673981/reports/intelligenthome</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Atilla</t>
+          <t>Atilla, Merisa</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Coupons, promo codes, Global Payouts</t>
+          <t>Property kolayxport.com, Türkiye time zone; Merisa needs viewer access</t>
         </is>
       </c>
     </row>
@@ -29938,17 +29972,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Reklam Kurulu influencer guide (send to partners)</t>
+          <t>YouTube Studio</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>https://ticaret.gov.tr/haberler/ticaret-bakanligi-sosyal-medya-etkileyicileri-icin-kilavuz-yayimladi</t>
+          <t>https://studio.youtube.com</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Merisa, Ekin</t>
+          <t>Atilla</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr"/>
@@ -29961,20 +29995,24 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Bionluk (freelancers)</t>
+          <t>Stripe dashboard (Tamsar, Inc.)</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>https://bionluk.com</t>
+          <t>https://dashboard.stripe.com</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Merisa</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr"/>
+          <t>Atilla</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Coupons, promo codes, Global Payouts</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -29984,38 +30022,70 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
+          <t>Reklam Kurulu influencer guide (send to partners)</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>https://ticaret.gov.tr/haberler/ticaret-bakanligi-sosyal-medya-etkileyicileri-icin-kilavuz-yayimladi</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Merisa, Ekin</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Bionluk (freelancers)</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>https://bionluk.com</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Merisa</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
           <t>PraPazar packages (pricing reference)</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C32" s="15" t="inlineStr">
         <is>
           <t>https://prapazar.com/tr/paketler</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Atilla</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
         <is>
           <t>Checked 2026-10-19</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="8" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -30219,6 +30289,20 @@
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n"/>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="4" t="n"/>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="8" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -30248,6 +30332,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -30259,7 +30345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30750,11 +30836,29 @@
       <c r="E23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
+      <c r="A24" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Tracking accounts created under kolayxport@gmail.com: GTM container GTM-N6SW5T7K (account KolayXport (Tamsar, Inc.)) and GA4 property G-V4ZC6HS65N; GTM v2 published with GA4 base + funnel-event tags</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Atilla (asked Claude to do it)</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>this session</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Google data-sharing options left off</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -31105,6 +31209,13 @@
       <c r="C74" s="4" t="n"/>
       <c r="D74" s="8" t="n"/>
       <c r="E74" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n"/>
+      <c r="B75" s="8" t="n"/>
+      <c r="C75" s="4" t="n"/>
+      <c r="D75" s="8" t="n"/>
+      <c r="E75" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>